<commit_message>
AI Specialist 별칭 누락 수정: NeurIPS/SIGKDD 등 7개 학회 오탐 해결
두 엑셀이 같은 학회를 다르게 적어서(nips vs NeurIPS, kdd vs SIGKDD 등)
ai_specialist=false로 잘못 표시되던 7개 학회를 AI_SPECIALIST_ALIASES 표로
바로잡는다. 이 중 5개(nips, kdd, mm, bigdataconf, siggrapha)는 노출 대상이라
사이트에 실제로 잘못된 배지가 보이고 있었다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgQHiBqjyZMvCHKWYf1dUT
</commit_message>
<xml_diff>
--- a/tests/fixtures/ai_specialist.xlsx
+++ b/tests/fixtures/ai_specialist.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E9"/>
+  <dimension ref="B2:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -525,6 +525,21 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="C10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SIGKDD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Knowledge Discovery and Data Mining</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>